<commit_message>
checkpoint before checking out main
</commit_message>
<xml_diff>
--- a/docs/clients/Investor_Generic_PV_BESS_1_5_10MW/cyprus-pv-bess-1-5-10mw-financial-model.xlsx
+++ b/docs/clients/Investor_Generic_PV_BESS_1_5_10MW/cyprus-pv-bess-1-5-10mw-financial-model.xlsx
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>INV-CY-PVBESS-1-5-10-2026 · July 2026 · Lighthief Cyprus Ltd · Non-binding indicative model</t>
+          <t>INV-CY-PVBESS-1-5-10-2026 · September 2026 · Lighthief Cyprus Ltd · Non-binding indicative model</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>1850</v>
+        <v>1800</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -647,7 +647,7 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Client-tested Year-1</t>
+          <t>Public SSOT — fixed bifacial</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>720000</v>
+        <v>600000</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>LH_EPC.pvPerMWp</t>
+          <t>Public turnkey EPC</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>15000</v>
+        <v>9000</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -687,7 +687,7 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>PV_DEFAULTS.omPerMWPerYear</t>
+          <t>Public PV O&amp;M</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>2450</v>
+        <v>2200</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -714,7 +714,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Client-tested Year-1</t>
+          <t>Public SSOT — 2P tracker bifacial</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>810000</v>
+        <v>780000</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>€720k + €90k/MW tracker adder (konia-epc-cost-model)</t>
+          <t>Public turnkey EPC</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>20000</v>
+        <v>9000</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>€15k × Konia tracker/fixed O&amp;M ratio</t>
+          <t>Public PV O&amp;M</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>0.874</v>
+        <v>0.95</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
@@ -821,7 +821,7 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Galascope 365-day 87.4%</t>
+          <t>Avdellero public capture 95%</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>140.88</v>
+        <v>151.38</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
@@ -888,7 +888,7 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>DAM.daytimeEURPerMWh 06–17h; full dataset €123.37</t>
+          <t>TSOC DAM 339-day sample 06–17h (to 4 Sep 2026)</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>210</v>
+        <v>212.42</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>market-data.json 18–21h avg Oct'25–Jul'26; winter €184</t>
+          <t>TSOC DAM 339-day sample evening peak</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>127000</v>
+        <v>125000</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>LH_EPC.bessPerMWh</t>
+          <t>4h LFP installed</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>350000</v>
+        <v>450000</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
@@ -955,7 +955,7 @@
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>constants INVESTMENT_SIZES</t>
+          <t>Public RTB acquisition</t>
         </is>
       </c>
     </row>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>0</v>
+        <v>150000</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
@@ -975,7 +975,7 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Site-specific; flexible teaser €80k/MW</t>
+          <t>Indicative EAC connection</t>
         </is>
       </c>
     </row>
@@ -1002,11 +1002,11 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>BESS LTSA Tier C (Yr 1–5)</t>
+          <t>BESS LTSA</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>1740</v>
+        <v>2200</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>LTSA.tierC.ratePerMWh</t>
+          <t>Public LTSA — all years (no OEM extended warranty in model)</t>
         </is>
       </c>
     </row>
@@ -1453,34 +1453,34 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Evening discharge €210</t>
+          <t>Evening discharge €212.42</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>market/data/market-data.json</t>
+          <t>lib/market/cyprus-tsoc-dam-sample.ts</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>18–21h avg Oct'25–Jul'26 (13,582 deduped prints)</t>
+          <t>339 TSOC DAM days to 4 Sep 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DAM daytime €140.88</t>
+          <t>DAM daytime €151.38</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>lib/deals/rtb-deal-types.ts → DAM</t>
+          <t>lib/market/cyprus-tsoc-dam-sample.ts</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>06–17h; full dataset 06–17h = €123.37</t>
+          <t>06:00–17:00 average</t>
         </is>
       </c>
     </row>
@@ -1492,109 +1492,109 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>rtb-deal-types.ts → BESS_DEFAULTS</t>
+          <t>lib/public-hybrid-ssot.ts</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>86.32% / 87.4% / 50%</t>
+          <t>86.32% / 95% / 50%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fixed PV EPC €720k/MWp</t>
+          <t>Fixed PV EPC €600k/MWp</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>rtb-deal-types.ts → LH_EPC.pvPerMWp</t>
+          <t>lib/public-hybrid-ssot.ts</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bifacial fixed, ~5MWp scale</t>
+          <t>Public turnkey EPC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tracker PV EPC €810k/MWp</t>
+          <t>Tracker PV EPC €780k/MWp</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>docs/internal/konia-epc-cost-model.md</t>
+          <t>lib/public-hybrid-ssot.ts</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>€720k + €90k/MW tracker adder</t>
+          <t>Public turnkey EPC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BESS EPC €127k/MWh</t>
+          <t>BESS EPC €125k/MWh</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>rtb-deal-types.ts → LH_EPC.bessPerMWh</t>
+          <t>lib/public-hybrid-ssot.ts</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tier-1 LFP installed</t>
+          <t>4h LFP installed</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PV O&amp;M €15k / €20k</t>
+          <t>PV O&amp;M €9k/MW/yr</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PV_DEFAULTS + konia O&amp;M ratio</t>
+          <t>lib/public-hybrid-ssot.ts</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fixed €15k; tracker +~35%</t>
+          <t>Public O&amp;M</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BESS LTSA €1,740/MWh/yr</t>
+          <t>BESS LTSA €2,200/MWh/yr</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>lib/portfolio-data.ts → LTSA.tierC</t>
+          <t>lib/public-hybrid-ssot.ts</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tier C, Yr 1–5</t>
+          <t>Public LTSA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RTB €350k/MW</t>
+          <t>RTB €450k/MW + connection €150k/MW</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>lib/constants.ts → INVESTMENT_SIZES</t>
+          <t>lib/public-hybrid-ssot.ts</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1668,7 +1668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1727,13 +1727,13 @@
         </is>
       </c>
       <c r="B6" s="17" t="n">
-        <v>1850</v>
+        <v>1800</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>1850</v>
+        <v>1800</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>1850</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="7">
@@ -1759,13 +1759,13 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>1578000</v>
+        <v>1700000</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>7890000</v>
+        <v>8500000</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>15780000</v>
+        <v>17000000</v>
       </c>
     </row>
     <row r="9">
@@ -1775,13 +1775,13 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>720000</v>
+        <v>600000</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>3600000</v>
+        <v>3000000</v>
       </c>
       <c r="D9" s="19" t="n">
-        <v>7200000</v>
+        <v>6000000</v>
       </c>
     </row>
     <row r="10">
@@ -1791,13 +1791,13 @@
         </is>
       </c>
       <c r="B10" s="19" t="n">
-        <v>508000</v>
+        <v>500000</v>
       </c>
       <c r="C10" s="19" t="n">
-        <v>2540000</v>
+        <v>2500000</v>
       </c>
       <c r="D10" s="19" t="n">
-        <v>5080000</v>
+        <v>5000000</v>
       </c>
     </row>
     <row r="11">
@@ -1807,13 +1807,13 @@
         </is>
       </c>
       <c r="B11" s="19" t="n">
-        <v>350000</v>
+        <v>450000</v>
       </c>
       <c r="C11" s="19" t="n">
-        <v>1750000</v>
+        <v>2250000</v>
       </c>
       <c r="D11" s="19" t="n">
-        <v>3500000</v>
+        <v>4500000</v>
       </c>
     </row>
     <row r="12">
@@ -1823,13 +1823,13 @@
         </is>
       </c>
       <c r="B12" s="19" t="n">
-        <v>1850</v>
+        <v>1800</v>
       </c>
       <c r="C12" s="19" t="n">
-        <v>9250</v>
+        <v>9000</v>
       </c>
       <c r="D12" s="19" t="n">
-        <v>18500</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="13">
@@ -1839,13 +1839,13 @@
         </is>
       </c>
       <c r="B13" s="19" t="n">
-        <v>276863.3484</v>
+        <v>293015.6071199999</v>
       </c>
       <c r="C13" s="19" t="n">
-        <v>1384316.742</v>
+        <v>1465078.0356</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>2768633.484</v>
+        <v>2930156.0712</v>
       </c>
     </row>
     <row r="14">
@@ -1855,13 +1855,13 @@
         </is>
       </c>
       <c r="B14" s="19" t="n">
-        <v>130314</v>
+        <v>136242</v>
       </c>
       <c r="C14" s="19" t="n">
-        <v>651570</v>
+        <v>681210</v>
       </c>
       <c r="D14" s="19" t="n">
-        <v>1303140</v>
+        <v>1362420</v>
       </c>
     </row>
     <row r="15">
@@ -1871,13 +1871,13 @@
         </is>
       </c>
       <c r="B15" s="19" t="n">
-        <v>146549.3484</v>
+        <v>156773.60712</v>
       </c>
       <c r="C15" s="19" t="n">
-        <v>732746.742</v>
+        <v>783868.0355999999</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>1465493.484</v>
+        <v>1567736.0712</v>
       </c>
     </row>
     <row r="16">
@@ -1887,13 +1887,13 @@
         </is>
       </c>
       <c r="B16" s="19" t="n">
-        <v>52850</v>
+        <v>49300</v>
       </c>
       <c r="C16" s="19" t="n">
-        <v>189250</v>
+        <v>171500</v>
       </c>
       <c r="D16" s="19" t="n">
-        <v>358500</v>
+        <v>323000</v>
       </c>
     </row>
     <row r="17">
@@ -1903,13 +1903,13 @@
         </is>
       </c>
       <c r="B17" s="19" t="n">
-        <v>196327.01356</v>
+        <v>214414.0464079999</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>1056635.0678</v>
+        <v>1147070.23204</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>2133270.1356</v>
+        <v>2314140.46408</v>
       </c>
     </row>
     <row r="18">
@@ -1919,13 +1919,13 @@
         </is>
       </c>
       <c r="B18" s="18" t="n">
-        <v>179587.961526</v>
+        <v>196501.9394468</v>
       </c>
       <c r="C18" s="18" t="n">
-        <v>961689.8076300001</v>
+        <v>1046259.697234</v>
       </c>
       <c r="D18" s="18" t="n">
-        <v>1940379.61526</v>
+        <v>2109519.394468</v>
       </c>
     </row>
     <row r="19">
@@ -1935,13 +1935,13 @@
         </is>
       </c>
       <c r="B19" s="20" t="n">
-        <v>0.1138073266958175</v>
+        <v>0.1155893761451764</v>
       </c>
       <c r="C19" s="20" t="n">
-        <v>0.1218871746045627</v>
+        <v>0.1230893761451765</v>
       </c>
       <c r="D19" s="20" t="n">
-        <v>0.1229644876590621</v>
+        <v>0.1240893761451765</v>
       </c>
     </row>
     <row r="20">
@@ -1951,13 +1951,13 @@
         </is>
       </c>
       <c r="B20" s="21" t="n">
-        <v>8.786780509068496</v>
+        <v>8.651314102984974</v>
       </c>
       <c r="C20" s="21" t="n">
-        <v>8.204308642351332</v>
+        <v>8.124177986088421</v>
       </c>
       <c r="D20" s="21" t="n">
-        <v>8.13242928131131</v>
+        <v>8.058707611117855</v>
       </c>
     </row>
     <row r="21">
@@ -1967,13 +1967,13 @@
         </is>
       </c>
       <c r="B21" s="21" t="n">
-        <v>9.663084565267889</v>
+        <v>9.309902527484178</v>
       </c>
       <c r="C21" s="21" t="n">
-        <v>8.892256088001579</v>
+        <v>8.65685939803625</v>
       </c>
       <c r="D21" s="21" t="n">
-        <v>8.800032192892999</v>
+        <v>8.577252168674477</v>
       </c>
     </row>
     <row r="22">
@@ -1983,13 +1983,13 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>0.07471869798819072</v>
+        <v>0.08094272556598039</v>
       </c>
       <c r="C22" s="20" t="n">
-        <v>0.08623128769760166</v>
+        <v>0.09128693095060202</v>
       </c>
       <c r="D22" s="20" t="n">
-        <v>0.08773177082434364</v>
+        <v>0.09264017355235069</v>
       </c>
     </row>
     <row r="23">
@@ -1999,19 +1999,19 @@
         </is>
       </c>
       <c r="B23" s="19" t="n">
-        <v>-56783.08520823169</v>
+        <v>11191.27189070395</v>
       </c>
       <c r="C23" s="19" t="n">
-        <v>341991.471183733</v>
+        <v>681863.2566784128</v>
       </c>
       <c r="D23" s="19" t="n">
-        <v>850891.4482941036</v>
+        <v>1530635.019283464</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>■ Configuration: Single-Axis Tracker · Bifacial · White Albedo</t>
+          <t>■ Configuration: Single-Axis Tracker · Bifacial 2P</t>
         </is>
       </c>
     </row>
@@ -2044,13 +2044,13 @@
         </is>
       </c>
       <c r="B28" s="17" t="n">
-        <v>2450</v>
+        <v>2200</v>
       </c>
       <c r="C28" s="17" t="n">
-        <v>2450</v>
+        <v>2200</v>
       </c>
       <c r="D28" s="17" t="n">
-        <v>2450</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="29">
@@ -2076,13 +2076,13 @@
         </is>
       </c>
       <c r="B30" s="18" t="n">
-        <v>1668000</v>
+        <v>1880000</v>
       </c>
       <c r="C30" s="18" t="n">
-        <v>8340000</v>
+        <v>9400000</v>
       </c>
       <c r="D30" s="18" t="n">
-        <v>16680000</v>
+        <v>18800000</v>
       </c>
     </row>
     <row r="31">
@@ -2092,13 +2092,13 @@
         </is>
       </c>
       <c r="B31" s="19" t="n">
-        <v>810000</v>
+        <v>780000</v>
       </c>
       <c r="C31" s="19" t="n">
-        <v>4050000</v>
+        <v>3900000</v>
       </c>
       <c r="D31" s="19" t="n">
-        <v>8100000</v>
+        <v>7800000</v>
       </c>
     </row>
     <row r="32">
@@ -2108,13 +2108,13 @@
         </is>
       </c>
       <c r="B32" s="19" t="n">
-        <v>508000</v>
+        <v>500000</v>
       </c>
       <c r="C32" s="19" t="n">
-        <v>2540000</v>
+        <v>2500000</v>
       </c>
       <c r="D32" s="19" t="n">
-        <v>5080000</v>
+        <v>5000000</v>
       </c>
     </row>
     <row r="33">
@@ -2124,13 +2124,13 @@
         </is>
       </c>
       <c r="B33" s="19" t="n">
-        <v>350000</v>
+        <v>450000</v>
       </c>
       <c r="C33" s="19" t="n">
-        <v>1750000</v>
+        <v>2250000</v>
       </c>
       <c r="D33" s="19" t="n">
-        <v>3500000</v>
+        <v>4500000</v>
       </c>
     </row>
     <row r="34">
@@ -2140,13 +2140,13 @@
         </is>
       </c>
       <c r="B34" s="19" t="n">
-        <v>2450</v>
+        <v>2200</v>
       </c>
       <c r="C34" s="19" t="n">
-        <v>12250</v>
+        <v>11000</v>
       </c>
       <c r="D34" s="19" t="n">
-        <v>24500</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="35">
@@ -2156,13 +2156,13 @@
         </is>
       </c>
       <c r="B35" s="19" t="n">
-        <v>366656.8668</v>
+        <v>358130.18648</v>
       </c>
       <c r="C35" s="19" t="n">
-        <v>1833284.334</v>
+        <v>1790650.9324</v>
       </c>
       <c r="D35" s="19" t="n">
-        <v>3666568.668</v>
+        <v>3581301.8648</v>
       </c>
     </row>
     <row r="36">
@@ -2172,13 +2172,13 @@
         </is>
       </c>
       <c r="B36" s="19" t="n">
-        <v>172578</v>
+        <v>166518</v>
       </c>
       <c r="C36" s="19" t="n">
-        <v>862890</v>
+        <v>832590</v>
       </c>
       <c r="D36" s="19" t="n">
-        <v>1725780</v>
+        <v>1665180</v>
       </c>
     </row>
     <row r="37">
@@ -2188,13 +2188,13 @@
         </is>
       </c>
       <c r="B37" s="19" t="n">
-        <v>194078.8668</v>
+        <v>191612.18648</v>
       </c>
       <c r="C37" s="19" t="n">
-        <v>970394.334</v>
+        <v>958060.9324</v>
       </c>
       <c r="D37" s="19" t="n">
-        <v>1940788.668</v>
+        <v>1916121.8648</v>
       </c>
     </row>
     <row r="38">
@@ -2204,13 +2204,13 @@
         </is>
       </c>
       <c r="B38" s="19" t="n">
-        <v>58300</v>
+        <v>50200</v>
       </c>
       <c r="C38" s="19" t="n">
-        <v>216500</v>
+        <v>176000</v>
       </c>
       <c r="D38" s="19" t="n">
-        <v>413000</v>
+        <v>332000</v>
       </c>
     </row>
     <row r="39">
@@ -2220,13 +2220,13 @@
         </is>
       </c>
       <c r="B39" s="19" t="n">
-        <v>271691.18012</v>
+        <v>272117.1678319999</v>
       </c>
       <c r="C39" s="19" t="n">
-        <v>1433455.9006</v>
+        <v>1435585.83916</v>
       </c>
       <c r="D39" s="19" t="n">
-        <v>2886911.8012</v>
+        <v>2891171.67832</v>
       </c>
     </row>
     <row r="40">
@@ -2236,13 +2236,13 @@
         </is>
       </c>
       <c r="B40" s="18" t="n">
-        <v>244322.503102</v>
+        <v>246899.5926571999</v>
       </c>
       <c r="C40" s="18" t="n">
-        <v>1285362.51551</v>
+        <v>1298247.963286</v>
       </c>
       <c r="D40" s="18" t="n">
-        <v>2587725.03102</v>
+        <v>2613495.926572</v>
       </c>
     </row>
     <row r="41">
@@ -2252,13 +2252,13 @@
         </is>
       </c>
       <c r="B41" s="20" t="n">
-        <v>0.1464763208045564</v>
+        <v>0.1313295705623404</v>
       </c>
       <c r="C41" s="20" t="n">
-        <v>0.1541202056966427</v>
+        <v>0.1381114854559574</v>
       </c>
       <c r="D41" s="20" t="n">
-        <v>0.1551393903489209</v>
+        <v>0.1390157407751064</v>
       </c>
     </row>
     <row r="42">
@@ -2268,13 +2268,13 @@
         </is>
       </c>
       <c r="B42" s="21" t="n">
-        <v>6.827042040018891</v>
+        <v>7.614431355543902</v>
       </c>
       <c r="C42" s="21" t="n">
-        <v>6.488441898191573</v>
+        <v>7.240527438385211</v>
       </c>
       <c r="D42" s="21" t="n">
-        <v>6.445816228560137</v>
+        <v>7.193429998821187</v>
       </c>
     </row>
     <row r="43">
@@ -2284,13 +2284,13 @@
         </is>
       </c>
       <c r="B43" s="21" t="n">
-        <v>7.274124944152986</v>
+        <v>8.093458694501351</v>
       </c>
       <c r="C43" s="21" t="n">
-        <v>6.860179215566277</v>
+        <v>7.646124604554445</v>
       </c>
       <c r="D43" s="21" t="n">
-        <v>6.809093091231898</v>
+        <v>7.590373567631153</v>
       </c>
     </row>
     <row r="44">
@@ -2300,13 +2300,13 @@
         </is>
       </c>
       <c r="B44" s="20" t="n">
-        <v>0.11528349859385</v>
+        <v>0.1005989900629649</v>
       </c>
       <c r="C44" s="20" t="n">
-        <v>0.1250874187080207</v>
+        <v>0.1094833725942626</v>
       </c>
       <c r="D44" s="20" t="n">
-        <v>0.1263769702354048</v>
+        <v>0.1106517461189106</v>
       </c>
     </row>
     <row r="45">
@@ -2316,13 +2316,13 @@
         </is>
       </c>
       <c r="B45" s="19" t="n">
-        <v>422422.9717922517</v>
+        <v>277537.5855559984</v>
       </c>
       <c r="C45" s="19" t="n">
-        <v>2738021.75618615</v>
+        <v>2013594.825004885</v>
       </c>
       <c r="D45" s="19" t="n">
-        <v>5642952.018298938</v>
+        <v>4194098.155936408</v>
       </c>
     </row>
     <row r="48">
@@ -2342,55 +2342,47 @@
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>Evening discharge €210/MWh = 18:00–21:00 average from market/data/market-data.json (Oct 2025–Jul 2026, deduped).</t>
+          <t>Evening discharge €212.42/MWh = TSOC DAM 339-day sample evening peak (1 Oct 2025–4 Sep 2026).</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Seasonality: winter (Oct–Feb) €179–194, spring (Mar–May) €240–260. Winter-only ≈ €184 as conservative sensitivity.</t>
+          <t>Fixed PV EPC €600k/MWp. Tracker €780k/MWp. RTB €450k/MW. EAC connection €150k/MW.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>Fixed PV EPC €720k/MWp (LH_EPC). Tracker €810k/MWp = €720k + €90k/MW adder (konia-epc-cost-model).</t>
+          <t>BESS EPC €125k/MWh installed 4h. LTSA €2,200/MWh/yr. PV O&amp;M €9k/MW/yr.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>BESS EPC €127k/MWh (LH_EPC). LTSA €1,740/MWh/yr (portfolio-data). PV O&amp;M €15k fixed / €20k tracker per MW/yr.</t>
+          <t>Cyprus rule: BESS cannot yet buy from DAM — no arbitrage. Capacity/ancillary = €0 (upside).</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>Cyprus rule: BESS cannot yet buy from DAM — no arbitrage. Capacity/ancillary = €0 (upside).</t>
+          <t>20y IRR/NPV include PV &amp; BESS degradation. OPEX is PV O&amp;M + BESS LTSA only (no OEM extended warranty). Indicative, non-binding, ex-VAT.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>20y IRR/NPV include PV &amp; BESS degradation and OEM extended warranty from Year 6. Indicative, non-binding, ex-VAT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
-        <is>
           <t>Contact: Alexander Papacosta, Cyprus Director · +357 99 164 158 · office@lighthief.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A56:D56"/>
+  <mergeCells count="9">
     <mergeCell ref="A53:D53"/>
     <mergeCell ref="A50:D50"/>
     <mergeCell ref="A4:D4"/>
@@ -2872,7 +2864,7 @@
         </is>
       </c>
       <c r="B47" s="26" t="n">
-        <v>179587.961526</v>
+        <v>196501.9394468</v>
       </c>
       <c r="C47" s="8">
         <f> B42 at default Inputs</f>
@@ -3351,7 +3343,7 @@
         </is>
       </c>
       <c r="B47" s="26" t="n">
-        <v>961689.8076300001</v>
+        <v>1046259.697234</v>
       </c>
       <c r="C47" s="8">
         <f> B42 at default Inputs</f>
@@ -3830,7 +3822,7 @@
         </is>
       </c>
       <c r="B47" s="26" t="n">
-        <v>1940379.61526</v>
+        <v>2109519.394468</v>
       </c>
       <c r="C47" s="8">
         <f> B42 at default Inputs</f>
@@ -3859,7 +3851,7 @@
     <row r="1">
       <c r="A1" s="22" t="inlineStr">
         <is>
-          <t>1 MW + 4 MWh · Single-Axis Tracker · Bifacial · White Albedo — live formulas (reads Inputs)</t>
+          <t>1 MW + 4 MWh · Single-Axis Tracker · Bifacial 2P — live formulas (reads Inputs)</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4301,7 @@
         </is>
       </c>
       <c r="B47" s="26" t="n">
-        <v>244322.503102</v>
+        <v>246899.5926571999</v>
       </c>
       <c r="C47" s="8">
         <f> B42 at default Inputs</f>
@@ -4338,7 +4330,7 @@
     <row r="1">
       <c r="A1" s="22" t="inlineStr">
         <is>
-          <t>5 MW + 20 MWh · Single-Axis Tracker · Bifacial · White Albedo — live formulas (reads Inputs)</t>
+          <t>5 MW + 20 MWh · Single-Axis Tracker · Bifacial 2P — live formulas (reads Inputs)</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4780,7 @@
         </is>
       </c>
       <c r="B47" s="26" t="n">
-        <v>1285362.51551</v>
+        <v>1298247.963286</v>
       </c>
       <c r="C47" s="8">
         <f> B42 at default Inputs</f>
@@ -4817,7 +4809,7 @@
     <row r="1">
       <c r="A1" s="22" t="inlineStr">
         <is>
-          <t>10 MW + 40 MWh · Single-Axis Tracker · Bifacial · White Albedo — live formulas (reads Inputs)</t>
+          <t>10 MW + 40 MWh · Single-Axis Tracker · Bifacial 2P — live formulas (reads Inputs)</t>
         </is>
       </c>
     </row>
@@ -5267,7 +5259,7 @@
         </is>
       </c>
       <c r="B47" s="26" t="n">
-        <v>2587725.03102</v>
+        <v>2613495.926572</v>
       </c>
       <c r="C47" s="8">
         <f> B42 at default Inputs</f>
@@ -5307,7 +5299,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Includes PV &amp; BESS degradation and OEM extended warranty from Year 6.</t>
+          <t>Includes PV &amp; BESS degradation. Recurring OPEX is PV O&amp;M + BESS LTSA only (OEM extended warranty excluded).</t>
         </is>
       </c>
     </row>
@@ -5355,22 +5347,22 @@
         </is>
       </c>
       <c r="B5" s="19" t="n">
-        <v>-1578000</v>
+        <v>-1700000</v>
       </c>
       <c r="C5" s="19" t="n">
-        <v>-7890000</v>
+        <v>-8500000</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>-15780000</v>
+        <v>-17000000</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>-1668000</v>
+        <v>-1880000</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>-8340000</v>
+        <v>-9400000</v>
       </c>
       <c r="G5" s="19" t="n">
-        <v>-16680000</v>
+        <v>-18800000</v>
       </c>
     </row>
     <row r="6">
@@ -5378,22 +5370,22 @@
         <v>1</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>179587.961526</v>
+        <v>196501.9394468</v>
       </c>
       <c r="C6" s="19" t="n">
-        <v>961689.8076300001</v>
+        <v>1046259.697234</v>
       </c>
       <c r="D6" s="19" t="n">
-        <v>1940379.61526</v>
+        <v>2109519.394468</v>
       </c>
       <c r="E6" s="19" t="n">
-        <v>244322.503102</v>
+        <v>246899.5926572</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>1285362.51551</v>
+        <v>1298247.963286</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>2587725.03102</v>
+        <v>2613495.926572</v>
       </c>
     </row>
     <row r="7">
@@ -5401,22 +5393,22 @@
         <v>2</v>
       </c>
       <c r="B7" s="19" t="n">
-        <v>176286.75418785</v>
+        <v>192982.5185606299</v>
       </c>
       <c r="C7" s="19" t="n">
-        <v>945183.77093925</v>
+        <v>1028662.59280315</v>
       </c>
       <c r="D7" s="19" t="n">
-        <v>1907367.5418785</v>
+        <v>2074325.1856063</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>239950.63392445</v>
+        <v>242598.07824077</v>
       </c>
       <c r="F7" s="19" t="n">
-        <v>1263503.16962225</v>
+        <v>1276740.39120385</v>
       </c>
       <c r="G7" s="19" t="n">
-        <v>2544006.3392445</v>
+        <v>2570480.7824077</v>
       </c>
     </row>
     <row r="8">
@@ -5424,22 +5416,22 @@
         <v>3</v>
       </c>
       <c r="B8" s="19" t="n">
-        <v>173058.1080121538</v>
+        <v>189540.6606836143</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>929040.5400607688</v>
+        <v>1011453.303418071</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>1875081.080121538</v>
+        <v>2039906.606836142</v>
       </c>
       <c r="E8" s="19" t="n">
-        <v>235674.8592593388</v>
+        <v>238391.3630577507</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>1242124.296296694</v>
+        <v>1255706.815288754</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>2501248.592593388</v>
+        <v>2528413.630577507</v>
       </c>
     </row>
     <row r="9">
@@ -5447,22 +5439,22 @@
         <v>4</v>
       </c>
       <c r="B9" s="19" t="n">
-        <v>169900.2588149549</v>
+        <v>186174.4788530889</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>913251.2940747746</v>
+        <v>994622.3942654446</v>
       </c>
       <c r="D9" s="19" t="n">
-        <v>1843502.588149549</v>
+        <v>2006244.788530889</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>231492.8427549403</v>
+        <v>234277.140820442</v>
       </c>
       <c r="F9" s="19" t="n">
-        <v>1221214.213774701</v>
+        <v>1235135.70410221</v>
       </c>
       <c r="G9" s="19" t="n">
-        <v>2459428.427549403</v>
+        <v>2487271.40820442</v>
       </c>
     </row>
     <row r="10">
@@ -5470,22 +5462,22 @@
         <v>5</v>
       </c>
       <c r="B10" s="19" t="n">
-        <v>166811.4862676705</v>
+        <v>182882.1330198938</v>
       </c>
       <c r="C10" s="19" t="n">
-        <v>897807.4313383525</v>
+        <v>978160.6650994691</v>
       </c>
       <c r="D10" s="19" t="n">
-        <v>1812614.862676705</v>
+        <v>1973321.330198938</v>
       </c>
       <c r="E10" s="19" t="n">
-        <v>227402.3061382664</v>
+        <v>230253.1625798703</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>1200761.530691332</v>
+        <v>1215015.812899351</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>2418523.061382663</v>
+        <v>2447031.625798702</v>
       </c>
     </row>
     <row r="11">
@@ -5493,22 +5485,22 @@
         <v>6</v>
       </c>
       <c r="B11" s="19" t="n">
-        <v>158140.4008019528</v>
+        <v>179661.828876838</v>
       </c>
       <c r="C11" s="19" t="n">
-        <v>854452.0040097638</v>
+        <v>962059.1443841902</v>
       </c>
       <c r="D11" s="19" t="n">
-        <v>1725904.008019528</v>
+        <v>1941118.28876838</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>217751.3157647482</v>
+        <v>226317.2352939131</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>1152506.578823741</v>
+        <v>1195336.176469566</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>2322013.157647482</v>
+        <v>2407672.352939131</v>
       </c>
     </row>
     <row r="12">
@@ -5516,22 +5508,22 @@
         <v>7</v>
       </c>
       <c r="B12" s="19" t="n">
-        <v>155184.7905419231</v>
+        <v>176511.8167164463</v>
       </c>
       <c r="C12" s="19" t="n">
-        <v>839673.9527096155</v>
+        <v>946309.0835822318</v>
       </c>
       <c r="D12" s="19" t="n">
-        <v>1696347.905419231</v>
+        <v>1909618.167164464</v>
       </c>
       <c r="E12" s="19" t="n">
-        <v>213837.1292041685</v>
+        <v>222467.2204312122</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>1132935.646020842</v>
+        <v>1176086.102156061</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>2282871.292041685</v>
+        <v>2369172.204312122</v>
       </c>
     </row>
     <row r="13">
@@ -5539,22 +5531,22 @@
         <v>8</v>
       </c>
       <c r="B13" s="19" t="n">
-        <v>152293.3482630941</v>
+        <v>173430.3903172568</v>
       </c>
       <c r="C13" s="19" t="n">
-        <v>825216.7413154707</v>
+        <v>930901.9515862844</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>1667433.482630941</v>
+        <v>1878803.903172569</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>210007.9218619354</v>
+        <v>218701.0326099806</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>1113789.609309677</v>
+        <v>1157255.163049903</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>2244579.218619354</v>
+        <v>2331510.326099806</v>
       </c>
     </row>
     <row r="14">
@@ -5562,22 +5554,22 @@
         <v>9</v>
       </c>
       <c r="B14" s="19" t="n">
-        <v>149464.5183773122</v>
+        <v>170415.8858579535</v>
       </c>
       <c r="C14" s="19" t="n">
-        <v>811072.591886561</v>
+        <v>915829.4292897675</v>
       </c>
       <c r="D14" s="19" t="n">
-        <v>1639145.183773122</v>
+        <v>1848658.858579535</v>
       </c>
       <c r="E14" s="19" t="n">
-        <v>206261.6336348188</v>
+        <v>215016.638270832</v>
       </c>
       <c r="F14" s="19" t="n">
-        <v>1095058.168174094</v>
+        <v>1138833.19135416</v>
       </c>
       <c r="G14" s="19" t="n">
-        <v>2207116.336348189</v>
+        <v>2294666.38270832</v>
       </c>
     </row>
     <row r="15">
@@ -5585,22 +5577,22 @@
         <v>10</v>
       </c>
       <c r="B15" s="19" t="n">
-        <v>146696.7839430709</v>
+        <v>167466.6808586395</v>
       </c>
       <c r="C15" s="19" t="n">
-        <v>797233.9197153543</v>
+        <v>901083.4042931977</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>1611467.839430709</v>
+        <v>1819166.808586395</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>202596.2556002831</v>
+        <v>211412.0543827817</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>1076731.278001415</v>
+        <v>1120810.271913908</v>
       </c>
       <c r="G15" s="19" t="n">
-        <v>2170462.556002831</v>
+        <v>2258620.543827817</v>
       </c>
     </row>
     <row r="16">
@@ -5608,22 +5600,22 @@
         <v>11</v>
       </c>
       <c r="B16" s="19" t="n">
-        <v>142553.7297005597</v>
+        <v>164581.1931485728</v>
       </c>
       <c r="C16" s="19" t="n">
-        <v>776518.6485027982</v>
+        <v>886655.9657428639</v>
       </c>
       <c r="D16" s="19" t="n">
-        <v>1570037.297005596</v>
+        <v>1790311.931485728</v>
       </c>
       <c r="E16" s="19" t="n">
-        <v>197574.892738579</v>
+        <v>207885.347181589</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>1051624.463692895</v>
+        <v>1103176.735907945</v>
       </c>
       <c r="G16" s="19" t="n">
-        <v>2120248.92738579</v>
+        <v>2223353.47181589</v>
       </c>
     </row>
     <row r="17">
@@ -5631,22 +5623,22 @@
         <v>12</v>
       </c>
       <c r="B17" s="19" t="n">
-        <v>139903.7851308308</v>
+        <v>161757.8798597007</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>763268.9256541542</v>
+        <v>872539.3992985035</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>1543537.851308308</v>
+        <v>1762078.798597007</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>194065.506686776</v>
+        <v>204434.6309396342</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>1034077.53343388</v>
+        <v>1085923.154698171</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>2085155.06686776</v>
+        <v>2188846.309396342</v>
       </c>
     </row>
     <row r="18">
@@ -5654,22 +5646,22 @@
         <v>13</v>
       </c>
       <c r="B18" s="19" t="n">
-        <v>137310.6075384814</v>
+        <v>158995.2364453512</v>
       </c>
       <c r="C18" s="19" t="n">
-        <v>750303.0376924067</v>
+        <v>858726.182226756</v>
       </c>
       <c r="D18" s="19" t="n">
-        <v>1517606.075384813</v>
+        <v>1734452.364453512</v>
       </c>
       <c r="E18" s="19" t="n">
-        <v>190631.2985239347</v>
+        <v>201058.0667665403</v>
       </c>
       <c r="F18" s="19" t="n">
-        <v>1016906.492619674</v>
+        <v>1069040.333832702</v>
       </c>
       <c r="G18" s="19" t="n">
-        <v>2050812.985239348</v>
+        <v>2155080.667665404</v>
       </c>
     </row>
     <row r="19">
@@ -5677,22 +5669,22 @@
         <v>14</v>
       </c>
       <c r="B19" s="19" t="n">
-        <v>134772.825157261</v>
+        <v>156291.7957234497</v>
       </c>
       <c r="C19" s="19" t="n">
-        <v>737614.1257863048</v>
+        <v>845208.9786172488</v>
       </c>
       <c r="D19" s="19" t="n">
-        <v>1492228.25157261</v>
+        <v>1707417.957234498</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>187270.4515866429</v>
+        <v>197753.861439772</v>
       </c>
       <c r="F19" s="19" t="n">
-        <v>1000102.257933215</v>
+        <v>1052519.30719886</v>
       </c>
       <c r="G19" s="19" t="n">
-        <v>2017204.51586643</v>
+        <v>2122038.61439772</v>
       </c>
     </row>
     <row r="20">
@@ -5700,22 +5692,22 @@
         <v>15</v>
       </c>
       <c r="B20" s="19" t="n">
-        <v>132289.1002780349</v>
+        <v>153646.1269436496</v>
       </c>
       <c r="C20" s="19" t="n">
-        <v>725195.5013901745</v>
+        <v>831980.6347182484</v>
       </c>
       <c r="D20" s="19" t="n">
-        <v>1467391.002780349</v>
+        <v>1680961.269436497</v>
       </c>
       <c r="E20" s="19" t="n">
-        <v>183981.1943141544</v>
+        <v>194520.2662644607</v>
       </c>
       <c r="F20" s="19" t="n">
-        <v>983655.971570772</v>
+        <v>1036351.331322304</v>
       </c>
       <c r="G20" s="19" t="n">
-        <v>1984311.943141544</v>
+        <v>2089702.662644607</v>
       </c>
     </row>
     <row r="21">
@@ -5723,22 +5715,22 @@
         <v>16</v>
       </c>
       <c r="B21" s="19" t="n">
-        <v>129858.128398541</v>
+        <v>151056.8348777781</v>
       </c>
       <c r="C21" s="19" t="n">
-        <v>713040.6419927048</v>
+        <v>819034.1743888907</v>
       </c>
       <c r="D21" s="19" t="n">
-        <v>1443081.28398541</v>
+        <v>1655068.348777781</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>180761.7991223921</v>
+        <v>191355.5759617288</v>
       </c>
       <c r="F21" s="19" t="n">
-        <v>967558.9956119605</v>
+        <v>1020527.879808644</v>
       </c>
       <c r="G21" s="19" t="n">
-        <v>1952117.991223921</v>
+        <v>2058055.759617288</v>
       </c>
     </row>
     <row r="22">
@@ -5746,22 +5738,22 @@
         <v>17</v>
       </c>
       <c r="B22" s="19" t="n">
-        <v>127478.6373943971</v>
+        <v>148522.5589330148</v>
       </c>
       <c r="C22" s="19" t="n">
-        <v>701143.1869719854</v>
+        <v>806362.794665074</v>
       </c>
       <c r="D22" s="19" t="n">
-        <v>1419286.373943971</v>
+        <v>1629725.589330148</v>
       </c>
       <c r="E22" s="19" t="n">
-        <v>177610.5813060934</v>
+        <v>188258.1275847958</v>
       </c>
       <c r="F22" s="19" t="n">
-        <v>951802.9065304672</v>
+        <v>1005040.637923979</v>
       </c>
       <c r="G22" s="19" t="n">
-        <v>1920605.813060935</v>
+        <v>2027081.275847958</v>
       </c>
     </row>
     <row r="23">
@@ -5769,22 +5761,22 @@
         <v>18</v>
       </c>
       <c r="B23" s="19" t="n">
-        <v>125149.3867108277</v>
+        <v>146041.9722872347</v>
       </c>
       <c r="C23" s="19" t="n">
-        <v>689496.9335541385</v>
+        <v>793959.8614361732</v>
       </c>
       <c r="D23" s="19" t="n">
-        <v>1395993.867108277</v>
+        <v>1604919.722872346</v>
       </c>
       <c r="E23" s="19" t="n">
-        <v>174525.8979683935</v>
+        <v>185226.2994621757</v>
       </c>
       <c r="F23" s="19" t="n">
-        <v>936379.4898419672</v>
+        <v>989881.4973108786</v>
       </c>
       <c r="G23" s="19" t="n">
-        <v>1889758.979683934</v>
+        <v>1996762.994621757</v>
       </c>
     </row>
     <row r="24">
@@ -5792,22 +5784,22 @@
         <v>19</v>
       </c>
       <c r="B24" s="19" t="n">
-        <v>122869.1665745911</v>
+        <v>143613.7810459613</v>
       </c>
       <c r="C24" s="19" t="n">
-        <v>678095.8328729557</v>
+        <v>781818.9052298063</v>
       </c>
       <c r="D24" s="19" t="n">
-        <v>1373191.665745911</v>
+        <v>1580637.810459613</v>
       </c>
       <c r="E24" s="19" t="n">
-        <v>171506.1469771612</v>
+        <v>182258.510167286</v>
       </c>
       <c r="F24" s="19" t="n">
-        <v>921280.7348858061</v>
+        <v>975042.55083643</v>
       </c>
       <c r="G24" s="19" t="n">
-        <v>1859561.469771612</v>
+        <v>1967085.10167286</v>
       </c>
     </row>
     <row r="25">
@@ -5815,22 +5807,22 @@
         <v>20</v>
       </c>
       <c r="B25" s="19" t="n">
-        <v>120636.7972256028</v>
+        <v>141236.7234203902</v>
       </c>
       <c r="C25" s="19" t="n">
-        <v>666933.9861280138</v>
+        <v>769933.617101951</v>
       </c>
       <c r="D25" s="19" t="n">
-        <v>1350867.972256028</v>
+        <v>1556867.234203902</v>
       </c>
       <c r="E25" s="19" t="n">
-        <v>168549.7659474199</v>
+        <v>179353.2175138102</v>
       </c>
       <c r="F25" s="19" t="n">
-        <v>906498.8297370994</v>
+        <v>960516.0875690513</v>
       </c>
       <c r="G25" s="19" t="n">
-        <v>1829997.659474199</v>
+        <v>1938032.175138103</v>
       </c>
     </row>
     <row r="27">
@@ -5840,22 +5832,22 @@
         </is>
       </c>
       <c r="B27" s="29" t="n">
-        <v>0.07471869798819072</v>
+        <v>0.08094272556598039</v>
       </c>
       <c r="C27" s="29" t="n">
-        <v>0.08623128769760166</v>
+        <v>0.09128693095060202</v>
       </c>
       <c r="D27" s="29" t="n">
-        <v>0.08773177082434364</v>
+        <v>0.09264017355235069</v>
       </c>
       <c r="E27" s="29" t="n">
-        <v>0.11528349859385</v>
+        <v>0.1005989900629649</v>
       </c>
       <c r="F27" s="29" t="n">
-        <v>0.1250874187080207</v>
+        <v>0.1094833725942626</v>
       </c>
       <c r="G27" s="29" t="n">
-        <v>0.1263769702354048</v>
+        <v>0.1106517461189106</v>
       </c>
     </row>
     <row r="28">
@@ -5865,22 +5857,22 @@
         </is>
       </c>
       <c r="B28" s="30" t="n">
-        <v>-56783.08520823169</v>
+        <v>11191.27189070395</v>
       </c>
       <c r="C28" s="30" t="n">
-        <v>341991.471183733</v>
+        <v>681863.2566784128</v>
       </c>
       <c r="D28" s="30" t="n">
-        <v>850891.4482941036</v>
+        <v>1530635.019283464</v>
       </c>
       <c r="E28" s="30" t="n">
-        <v>422422.9717922517</v>
+        <v>277537.5855559984</v>
       </c>
       <c r="F28" s="30" t="n">
-        <v>2738021.75618615</v>
+        <v>2013594.825004885</v>
       </c>
       <c r="G28" s="30" t="n">
-        <v>5642952.018298938</v>
+        <v>4194098.155936408</v>
       </c>
     </row>
     <row r="29">
@@ -5890,22 +5882,22 @@
         </is>
       </c>
       <c r="B29" s="31" t="n">
-        <v>8.786780509068496</v>
+        <v>8.651314102984974</v>
       </c>
       <c r="C29" s="31" t="n">
-        <v>8.204308642351332</v>
+        <v>8.124177986088421</v>
       </c>
       <c r="D29" s="31" t="n">
-        <v>8.13242928131131</v>
+        <v>8.058707611117855</v>
       </c>
       <c r="E29" s="31" t="n">
-        <v>6.827042040018891</v>
+        <v>7.614431355543902</v>
       </c>
       <c r="F29" s="31" t="n">
-        <v>6.488441898191573</v>
+        <v>7.240527438385211</v>
       </c>
       <c r="G29" s="31" t="n">
-        <v>6.445816228560137</v>
+        <v>7.193429998821187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>